<commit_message>
DigitalLED V0.2: 1.2 kOhm opto-triac series resistor, measured bus current
The IL4118 opto-triac needs far less trigger current than the MOC3043
the 270 Ohm resistor was sized for (I_FT max 1.3 mA vs. 5 mA). R4 is now
1.2 kOhm (~1.75 mA LED current at 3.3 V, C22765); the mains stage
switches reliably with it.

Bus current measured at the nominal 16 V: 1.67 mA with the LED supply
off and 2.6 mA while it is on. The README now states the measured value
instead of the earlier estimate.
</commit_message>
<xml_diff>
--- a/Hardware/DALI_Load_250W_DigitalLED/JLC_PCBA_BOM-DALI_LOAD_DigitalLED(V0.2).xlsx
+++ b/Hardware/DALI_Load_250W_DigitalLED/JLC_PCBA_BOM-DALI_LOAD_DigitalLED(V0.2).xlsx
@@ -1257,7 +1257,7 @@
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>1.2k</t>
         </is>
       </c>
       <c r="B21" s="24" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>C22966</t>
+          <t>C22765</t>
         </is>
       </c>
     </row>

</xml_diff>